<commit_message>
Fix Persian TextLine crash + submodule update
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tppc_lims_master/TPPC_SENAITE_Setup.xlsx
+++ b/outputs/tppc_lims_master/TPPC_SENAITE_Setup.xlsx
@@ -7683,78 +7683,78 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>آزمون‌های آب و محلول</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Water Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>نفت خام</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>ضدیخ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>ضدیخ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>قیر</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>قیر</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>گریس</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>گریس</t>
         </is>
       </c>
     </row>
@@ -8253,12 +8253,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -8329,12 +8329,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -8405,12 +8405,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -8481,12 +8481,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -8553,12 +8553,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>قیر</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>قیر</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -8625,12 +8625,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -8697,12 +8697,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -8773,12 +8773,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -8849,12 +8849,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -8925,12 +8925,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -9001,12 +9001,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -9077,12 +9077,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -9153,12 +9153,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -9229,12 +9229,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -9305,12 +9305,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -9381,12 +9381,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -9457,12 +9457,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -9533,12 +9533,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -9609,12 +9609,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -9685,12 +9685,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -9761,12 +9761,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>ضدیخ</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>ضدیخ</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -9837,12 +9837,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -9913,12 +9913,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -9989,12 +9989,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -10065,12 +10065,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -10141,12 +10141,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -10217,12 +10217,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -10293,12 +10293,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -10369,12 +10369,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -10445,12 +10445,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -10521,12 +10521,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -10597,12 +10597,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -10673,12 +10673,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -10749,12 +10749,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -10825,12 +10825,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -10901,12 +10901,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -10977,12 +10977,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -11053,12 +11053,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -11129,12 +11129,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -11205,12 +11205,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -11281,12 +11281,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -11357,12 +11357,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -11433,12 +11433,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -11509,12 +11509,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -11585,12 +11585,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -11661,12 +11661,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -11737,12 +11737,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
@@ -11813,12 +11813,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -11889,12 +11889,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -11965,12 +11965,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -12041,12 +12041,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -12117,12 +12117,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -12193,12 +12193,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
@@ -12269,12 +12269,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -12345,12 +12345,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>آزمون‌های آب و محلول</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Water Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -12421,12 +12421,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -12497,12 +12497,12 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -12573,12 +12573,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -12649,12 +12649,12 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
@@ -12725,12 +12725,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
@@ -12801,12 +12801,12 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
@@ -12877,12 +12877,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -12953,12 +12953,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
@@ -13029,12 +13029,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -13105,12 +13105,12 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
@@ -13181,12 +13181,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -13257,12 +13257,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
@@ -13333,12 +13333,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -13409,12 +13409,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
@@ -13485,12 +13485,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -13561,12 +13561,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -13637,12 +13637,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -13713,12 +13713,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
@@ -13789,12 +13789,12 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -13865,12 +13865,12 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
@@ -13941,12 +13941,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -14017,12 +14017,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
@@ -14093,12 +14093,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H81" t="inlineStr"/>
@@ -14169,12 +14169,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -14245,12 +14245,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -14321,12 +14321,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -14397,12 +14397,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -14473,12 +14473,12 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
@@ -14549,12 +14549,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -14625,12 +14625,12 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
@@ -14701,12 +14701,12 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -14777,12 +14777,12 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
@@ -14853,12 +14853,12 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
@@ -14929,12 +14929,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
@@ -15005,12 +15005,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
@@ -15081,12 +15081,12 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
@@ -15157,12 +15157,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
@@ -15233,12 +15233,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H96" t="inlineStr"/>
@@ -15309,12 +15309,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H97" t="inlineStr"/>
@@ -15385,12 +15385,12 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H98" t="inlineStr"/>
@@ -15461,12 +15461,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H99" t="inlineStr"/>
@@ -15537,12 +15537,12 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
@@ -15613,12 +15613,12 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -15689,12 +15689,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
@@ -15765,12 +15765,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
@@ -15841,12 +15841,12 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
@@ -15917,12 +15917,12 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>عناصر و فلزات (ICP)</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -15993,12 +15993,12 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H106" t="inlineStr"/>
@@ -16069,12 +16069,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>ضدیخ</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>ضدیخ</t>
         </is>
       </c>
       <c r="H107" t="inlineStr"/>
@@ -16145,12 +16145,12 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
@@ -16217,12 +16217,12 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -16293,12 +16293,12 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -16369,12 +16369,12 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H111" t="inlineStr"/>
@@ -16445,12 +16445,12 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -16521,12 +16521,12 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
@@ -16597,12 +16597,12 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H114" t="inlineStr"/>
@@ -16673,12 +16673,12 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -16749,12 +16749,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
@@ -16825,12 +16825,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
@@ -16901,12 +16901,12 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>قیر</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>قیر</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -16977,12 +16977,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -17053,12 +17053,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H120" t="inlineStr"/>
@@ -17129,12 +17129,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>آزمون‌های آب و محلول</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Water Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -17205,12 +17205,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -17281,12 +17281,12 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
@@ -17357,12 +17357,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H124" t="inlineStr"/>
@@ -17433,12 +17433,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H125" t="inlineStr"/>
@@ -17509,12 +17509,12 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H126" t="inlineStr"/>
@@ -17585,12 +17585,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H127" t="inlineStr"/>
@@ -17661,12 +17661,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H128" t="inlineStr"/>
@@ -17737,12 +17737,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -17813,12 +17813,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -17889,12 +17889,12 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -17965,12 +17965,12 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
@@ -18041,12 +18041,12 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
@@ -18117,12 +18117,12 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
@@ -18193,12 +18193,12 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H135" t="inlineStr"/>
@@ -18269,12 +18269,12 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
@@ -18345,12 +18345,12 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H137" t="inlineStr"/>
@@ -18421,12 +18421,12 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
@@ -18497,12 +18497,12 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>تیتراسیون و محتوای آب</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -18573,12 +18573,12 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>دستگاهی و کروماتوگرافی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
@@ -18649,12 +18649,12 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
@@ -18721,12 +18721,12 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
@@ -18797,12 +18797,12 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
@@ -18873,12 +18873,12 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
@@ -18949,12 +18949,12 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="H145" t="inlineStr"/>
@@ -19025,12 +19025,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="H146" t="inlineStr"/>
@@ -19101,12 +19101,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H147" t="inlineStr"/>
@@ -19177,12 +19177,12 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H148" t="inlineStr"/>
@@ -19253,12 +19253,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H149" t="inlineStr"/>
@@ -19329,12 +19329,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
@@ -19405,12 +19405,12 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H151" t="inlineStr"/>
@@ -19477,12 +19477,12 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>متفرقه</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H152" t="inlineStr"/>
@@ -19553,12 +19553,12 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H153" t="inlineStr"/>
@@ -19629,12 +19629,12 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H154" t="inlineStr"/>
@@ -19705,12 +19705,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H155" t="inlineStr"/>
@@ -19781,12 +19781,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H156" t="inlineStr"/>
@@ -19857,12 +19857,12 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H157" t="inlineStr"/>
@@ -19933,12 +19933,12 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H158" t="inlineStr"/>
@@ -20009,12 +20009,12 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H159" t="inlineStr"/>
@@ -20085,12 +20085,12 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H160" t="inlineStr"/>
@@ -20161,12 +20161,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>خواص فیزیکی</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="H161" t="inlineStr"/>
@@ -20598,7 +20598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20645,7 +20645,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oil Lab</t>
+          <t>هیدروکربن</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -20654,7 +20654,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Water Lab</t>
+          <t>روغن</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -20663,11 +20663,38 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Instrumental</t>
+          <t>نفت خام</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ضدیخ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>قیر</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>گریس</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20725,7 +20752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20808,6 +20835,223 @@
           <t>error</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>اندازه گیری میزان خاکستر برحسب درصد وزنی</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>تعیین رنگ بر اساس مقیاس ASTM</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>اندازه گیری نقطه اشتعال با دستگاه سربسته پنسکی مارتنز</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>55</v>
+      </c>
+      <c r="F6" t="n">
+        <v>999999</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>گرانروی در 40 درجه سانتی گراد</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>اندازه گیری آب از طریق تیتراسیون کارل فیشر(کولومتری)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>اندازه گیری چگالی،چگالی نسبی یا گراویتی API با استفاده از روش هیدرومتر</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>820</v>
+      </c>
+      <c r="F9" t="n">
+        <v>845</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>محاسبه شاخص ستان سوخت های حاصل از بخش میانی برج تقطیر به روش معادله چهار متغیره</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>46</v>
+      </c>
+      <c r="F10" t="n">
+        <v>999999</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>تشخیص خوردگی تیغه مسی</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>نفت گاز</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>اندازه گیری نقطه اشتعال با دستگاه سربسته پنسکى مارتنز</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>55</v>
+      </c>
+      <c r="F12" t="n">
+        <v>999999</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>